<commit_message>
Doubly linked list and refactor
</commit_message>
<xml_diff>
--- a/src/DSA patterns Cheat Sheet.xlsx
+++ b/src/DSA patterns Cheat Sheet.xlsx
@@ -1447,13 +1447,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1471,6 +1464,13 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1654,7 +1654,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="43">
+  <fills count="44">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1677,6 +1677,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF00FF00"/>
         <bgColor rgb="FF00FF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -2053,7 +2059,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2077,16 +2083,16 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -2095,89 +2101,89 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2199,26 +2205,28 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
@@ -2774,7 +2782,7 @@
       <c r="D6" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="15" t="s">
         <v>14</v>
       </c>
     </row>
@@ -2783,7 +2791,7 @@
       <c r="B7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="16" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="8"/>
@@ -2794,7 +2802,7 @@
       <c r="B8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="17" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="8"/>
@@ -2805,7 +2813,7 @@
       <c r="B9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="17" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="8"/>
@@ -2816,7 +2824,7 @@
       <c r="B10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="17" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="8"/>
@@ -2827,7 +2835,7 @@
       <c r="B11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="17" t="s">
         <v>24</v>
       </c>
       <c r="D11" s="8"/>
@@ -2838,7 +2846,7 @@
       <c r="B12" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="17" t="s">
         <v>26</v>
       </c>
       <c r="D12" s="8"/>
@@ -2846,10 +2854,10 @@
     </row>
     <row r="13" customHeight="1" spans="1:5">
       <c r="A13" s="6"/>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="17" t="s">
         <v>28</v>
       </c>
       <c r="D13" s="8"/>
@@ -2860,7 +2868,7 @@
       <c r="B14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="17" t="s">
         <v>30</v>
       </c>
       <c r="D14" s="8"/>
@@ -2871,10 +2879,10 @@
       <c r="B15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="17" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2892,7 +2900,7 @@
       <c r="B17" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="17" t="s">
         <v>36</v>
       </c>
       <c r="D17" s="8"/>
@@ -2903,7 +2911,7 @@
       <c r="B18" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="17" t="s">
         <v>38</v>
       </c>
       <c r="D18" s="8"/>
@@ -2914,7 +2922,7 @@
       <c r="B19" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="17" t="s">
         <v>40</v>
       </c>
       <c r="D19" s="8"/>
@@ -2925,7 +2933,7 @@
       <c r="B20" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="17" t="s">
         <v>42</v>
       </c>
       <c r="D20" s="8"/>
@@ -2936,7 +2944,7 @@
       <c r="B21" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="17" t="s">
         <v>44</v>
       </c>
       <c r="D21" s="8"/>
@@ -2947,7 +2955,7 @@
       <c r="B22" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="17" t="s">
         <v>46</v>
       </c>
       <c r="D22" s="8"/>
@@ -2958,7 +2966,7 @@
       <c r="B23" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="17" t="s">
         <v>48</v>
       </c>
       <c r="D23" s="8"/>
@@ -2969,7 +2977,7 @@
       <c r="B24" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="17" t="s">
         <v>50</v>
       </c>
       <c r="D24" s="8"/>
@@ -2989,7 +2997,7 @@
       <c r="B26" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="19" t="s">
         <v>53</v>
       </c>
       <c r="D26" s="8"/>
@@ -3000,7 +3008,7 @@
       <c r="B27" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="17" t="s">
         <v>55</v>
       </c>
       <c r="D27" s="8"/>
@@ -3011,7 +3019,7 @@
       <c r="B28" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="17" t="s">
         <v>57</v>
       </c>
       <c r="D28" s="8"/>
@@ -3022,7 +3030,7 @@
       <c r="B29" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="17" t="s">
         <v>59</v>
       </c>
       <c r="D29" s="8"/>
@@ -3033,7 +3041,7 @@
       <c r="B30" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="17" t="s">
         <v>61</v>
       </c>
       <c r="D30" s="8"/>
@@ -3044,7 +3052,7 @@
       <c r="B31" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="17" t="s">
         <v>63</v>
       </c>
       <c r="D31" s="8"/>
@@ -3055,7 +3063,7 @@
       <c r="B32" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="17" t="s">
         <v>65</v>
       </c>
       <c r="D32" s="8"/>
@@ -3066,7 +3074,7 @@
       <c r="B33" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="C33" s="17" t="s">
         <v>55</v>
       </c>
       <c r="D33" s="8"/>
@@ -3077,7 +3085,7 @@
       <c r="B34" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="17" t="s">
         <v>68</v>
       </c>
       <c r="D34" s="8"/>
@@ -3088,7 +3096,7 @@
       <c r="B35" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="C35" s="17" t="s">
         <v>70</v>
       </c>
       <c r="D35" s="8"/>
@@ -3099,7 +3107,7 @@
       <c r="B36" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="17" t="s">
         <v>72</v>
       </c>
       <c r="D36" s="8"/>
@@ -3110,7 +3118,7 @@
       <c r="B37" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="15" t="s">
+      <c r="C37" s="16" t="s">
         <v>74</v>
       </c>
       <c r="D37" s="8"/>
@@ -3127,10 +3135,10 @@
     </row>
     <row r="39" customHeight="1" spans="1:5">
       <c r="A39" s="6"/>
-      <c r="B39" s="18" t="s">
+      <c r="B39" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="C39" s="17" t="s">
+      <c r="C39" s="19" t="s">
         <v>77</v>
       </c>
       <c r="D39" s="8"/>
@@ -3141,7 +3149,7 @@
       <c r="B40" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="17" t="s">
+      <c r="C40" s="19" t="s">
         <v>79</v>
       </c>
       <c r="D40" s="8"/>
@@ -3149,10 +3157,10 @@
     </row>
     <row r="41" customHeight="1" spans="1:5">
       <c r="A41" s="6"/>
-      <c r="B41" s="18" t="s">
+      <c r="B41" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="C41" s="19" t="s">
         <v>81</v>
       </c>
       <c r="D41" s="8"/>
@@ -3160,10 +3168,10 @@
     </row>
     <row r="42" customHeight="1" spans="1:5">
       <c r="A42" s="6"/>
-      <c r="B42" s="18" t="s">
+      <c r="B42" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="C42" s="17" t="s">
+      <c r="C42" s="19" t="s">
         <v>83</v>
       </c>
       <c r="D42" s="8"/>
@@ -3171,10 +3179,10 @@
     </row>
     <row r="43" customHeight="1" spans="1:5">
       <c r="A43" s="6"/>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="C43" s="17" t="s">
+      <c r="C43" s="19" t="s">
         <v>85</v>
       </c>
       <c r="D43" s="8"/>
@@ -3182,10 +3190,10 @@
     </row>
     <row r="44" customHeight="1" spans="1:5">
       <c r="A44" s="6"/>
-      <c r="B44" s="18" t="s">
+      <c r="B44" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="C44" s="17" t="s">
+      <c r="C44" s="19" t="s">
         <v>87</v>
       </c>
       <c r="D44" s="8"/>
@@ -3202,10 +3210,10 @@
     </row>
     <row r="46" customHeight="1" spans="1:5">
       <c r="A46" s="6"/>
-      <c r="B46" s="18" t="s">
+      <c r="B46" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="C46" s="17" t="s">
+      <c r="C46" s="19" t="s">
         <v>90</v>
       </c>
       <c r="D46" s="8"/>
@@ -3213,10 +3221,10 @@
     </row>
     <row r="47" customHeight="1" spans="1:5">
       <c r="A47" s="6"/>
-      <c r="B47" s="18" t="s">
+      <c r="B47" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="C47" s="17" t="s">
+      <c r="C47" s="19" t="s">
         <v>92</v>
       </c>
       <c r="D47" s="8"/>
@@ -3224,10 +3232,10 @@
     </row>
     <row r="48" customHeight="1" spans="1:5">
       <c r="A48" s="6"/>
-      <c r="B48" s="18" t="s">
+      <c r="B48" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="C48" s="17" t="s">
+      <c r="C48" s="19" t="s">
         <v>94</v>
       </c>
       <c r="D48" s="8"/>
@@ -3235,10 +3243,10 @@
     </row>
     <row r="49" customHeight="1" spans="1:5">
       <c r="A49" s="6"/>
-      <c r="B49" s="18" t="s">
+      <c r="B49" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="C49" s="17" t="s">
+      <c r="C49" s="19" t="s">
         <v>96</v>
       </c>
       <c r="D49" s="8"/>
@@ -3246,10 +3254,10 @@
     </row>
     <row r="50" customHeight="1" spans="1:5">
       <c r="A50" s="6"/>
-      <c r="B50" s="19" t="s">
+      <c r="B50" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="C50" s="17" t="s">
+      <c r="C50" s="19" t="s">
         <v>98</v>
       </c>
       <c r="D50" s="8"/>
@@ -3257,10 +3265,10 @@
     </row>
     <row r="51" customHeight="1" spans="1:5">
       <c r="A51" s="6"/>
-      <c r="B51" s="19" t="s">
+      <c r="B51" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="C51" s="17" t="s">
+      <c r="C51" s="19" t="s">
         <v>100</v>
       </c>
       <c r="D51" s="8"/>
@@ -3280,7 +3288,7 @@
       <c r="B53" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="C53" s="11" t="s">
+      <c r="C53" s="17" t="s">
         <v>103</v>
       </c>
       <c r="D53" s="8"/>
@@ -3291,7 +3299,7 @@
       <c r="B54" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="C54" s="11" t="s">
+      <c r="C54" s="17" t="s">
         <v>105</v>
       </c>
       <c r="D54" s="8"/>
@@ -3302,7 +3310,7 @@
       <c r="B55" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C55" s="11" t="s">
+      <c r="C55" s="17" t="s">
         <v>107</v>
       </c>
       <c r="D55" s="8"/>
@@ -3313,7 +3321,7 @@
       <c r="B56" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="C56" s="11" t="s">
+      <c r="C56" s="17" t="s">
         <v>109</v>
       </c>
       <c r="E56" s="8"/>
@@ -3323,7 +3331,7 @@
       <c r="B57" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="C57" s="11" t="s">
+      <c r="C57" s="17" t="s">
         <v>111</v>
       </c>
       <c r="D57" s="8"/>
@@ -3334,7 +3342,7 @@
       <c r="B58" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="C58" s="11" t="s">
+      <c r="C58" s="17" t="s">
         <v>113</v>
       </c>
       <c r="D58" s="8"/>
@@ -3345,7 +3353,7 @@
       <c r="B59" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C59" s="11" t="s">
+      <c r="C59" s="17" t="s">
         <v>115</v>
       </c>
       <c r="D59" s="8"/>
@@ -3365,7 +3373,7 @@
       <c r="B61" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="C61" s="11" t="s">
+      <c r="C61" s="17" t="s">
         <v>118</v>
       </c>
       <c r="D61" s="8"/>
@@ -3376,7 +3384,7 @@
       <c r="B62" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="C62" s="11" t="s">
+      <c r="C62" s="17" t="s">
         <v>120</v>
       </c>
       <c r="D62" s="8"/>
@@ -3387,7 +3395,7 @@
       <c r="B63" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C63" s="11" t="s">
+      <c r="C63" s="17" t="s">
         <v>122</v>
       </c>
       <c r="D63" s="8"/>
@@ -3398,7 +3406,7 @@
       <c r="B64" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="C64" s="11" t="s">
+      <c r="C64" s="17" t="s">
         <v>124</v>
       </c>
       <c r="D64" s="8"/>
@@ -3409,7 +3417,7 @@
       <c r="B65" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C65" s="11" t="s">
+      <c r="C65" s="17" t="s">
         <v>126</v>
       </c>
       <c r="D65" s="8"/>
@@ -3420,7 +3428,7 @@
       <c r="B66" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="C66" s="11" t="s">
+      <c r="C66" s="17" t="s">
         <v>128</v>
       </c>
       <c r="D66" s="8"/>
@@ -3437,10 +3445,10 @@
     </row>
     <row r="68" customHeight="1" spans="1:5">
       <c r="A68" s="6"/>
-      <c r="B68" s="20" t="s">
+      <c r="B68" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="C68" s="11" t="s">
+      <c r="C68" s="17" t="s">
         <v>131</v>
       </c>
       <c r="D68" s="8"/>
@@ -3451,7 +3459,7 @@
       <c r="B69" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="C69" s="11" t="s">
+      <c r="C69" s="17" t="s">
         <v>133</v>
       </c>
       <c r="D69" s="8"/>
@@ -3471,7 +3479,7 @@
       <c r="B71" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="C71" s="11" t="s">
+      <c r="C71" s="17" t="s">
         <v>136</v>
       </c>
       <c r="D71" s="13"/>
@@ -3482,7 +3490,7 @@
       <c r="B72" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="C72" s="11" t="s">
+      <c r="C72" s="17" t="s">
         <v>138</v>
       </c>
       <c r="D72" s="8"/>
@@ -3493,7 +3501,7 @@
       <c r="B73" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C73" s="11" t="s">
+      <c r="C73" s="17" t="s">
         <v>140</v>
       </c>
       <c r="D73" s="8"/>
@@ -3504,7 +3512,7 @@
       <c r="B74" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="C74" s="11" t="s">
+      <c r="C74" s="17" t="s">
         <v>142</v>
       </c>
       <c r="D74" s="8"/>
@@ -3515,7 +3523,7 @@
       <c r="B75" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C75" s="11" t="s">
+      <c r="C75" s="17" t="s">
         <v>144</v>
       </c>
       <c r="D75" s="8"/>
@@ -3526,7 +3534,7 @@
       <c r="B76" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="C76" s="11" t="s">
+      <c r="C76" s="17" t="s">
         <v>146</v>
       </c>
       <c r="D76" s="8"/>
@@ -3546,7 +3554,7 @@
       <c r="B78" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="C78" s="11" t="s">
+      <c r="C78" s="17" t="s">
         <v>149</v>
       </c>
       <c r="D78" s="8"/>
@@ -3557,7 +3565,7 @@
       <c r="B79" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="C79" s="11" t="s">
+      <c r="C79" s="17" t="s">
         <v>151</v>
       </c>
       <c r="D79" s="8"/>
@@ -3568,7 +3576,7 @@
       <c r="B80" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="C80" s="11" t="s">
+      <c r="C80" s="17" t="s">
         <v>153</v>
       </c>
       <c r="D80" s="8"/>
@@ -3579,7 +3587,7 @@
       <c r="B81" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="C81" s="11" t="s">
+      <c r="C81" s="17" t="s">
         <v>155</v>
       </c>
       <c r="D81" s="8"/>
@@ -3590,7 +3598,7 @@
       <c r="B82" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="C82" s="21"/>
+      <c r="C82" s="23"/>
       <c r="D82" s="8"/>
       <c r="E82" s="8"/>
     </row>
@@ -3599,7 +3607,7 @@
       <c r="B83" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="C83" s="11" t="s">
+      <c r="C83" s="17" t="s">
         <v>158</v>
       </c>
       <c r="D83" s="8"/>
@@ -3610,7 +3618,7 @@
       <c r="B84" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="C84" s="11" t="s">
+      <c r="C84" s="17" t="s">
         <v>160</v>
       </c>
       <c r="D84" s="8"/>
@@ -3621,7 +3629,7 @@
       <c r="B85" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="C85" s="11" t="s">
+      <c r="C85" s="17" t="s">
         <v>162</v>
       </c>
       <c r="D85" s="8"/>
@@ -3632,7 +3640,7 @@
       <c r="B86" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="C86" s="11" t="s">
+      <c r="C86" s="17" t="s">
         <v>164</v>
       </c>
       <c r="D86" s="8"/>
@@ -3643,7 +3651,7 @@
       <c r="B87" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="C87" s="11" t="s">
+      <c r="C87" s="17" t="s">
         <v>166</v>
       </c>
       <c r="D87" s="8"/>
@@ -3654,7 +3662,7 @@
       <c r="B88" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="C88" s="11" t="s">
+      <c r="C88" s="17" t="s">
         <v>168</v>
       </c>
       <c r="D88" s="8"/>
@@ -3665,7 +3673,7 @@
       <c r="B89" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="C89" s="11" t="s">
+      <c r="C89" s="17" t="s">
         <v>170</v>
       </c>
       <c r="D89" s="8"/>
@@ -3676,7 +3684,7 @@
       <c r="B90" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C90" s="11" t="s">
+      <c r="C90" s="17" t="s">
         <v>172</v>
       </c>
       <c r="D90" s="8"/>
@@ -3687,7 +3695,7 @@
       <c r="B91" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="C91" s="11" t="s">
+      <c r="C91" s="17" t="s">
         <v>174</v>
       </c>
       <c r="D91" s="8"/>
@@ -3698,7 +3706,7 @@
       <c r="B92" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="C92" s="11" t="s">
+      <c r="C92" s="17" t="s">
         <v>176</v>
       </c>
       <c r="D92" s="8"/>
@@ -3709,7 +3717,7 @@
       <c r="B93" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="C93" s="11" t="s">
+      <c r="C93" s="17" t="s">
         <v>178</v>
       </c>
       <c r="D93" s="8"/>
@@ -3720,7 +3728,7 @@
       <c r="B94" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C94" s="11" t="s">
+      <c r="C94" s="17" t="s">
         <v>180</v>
       </c>
       <c r="D94" s="8"/>
@@ -3731,7 +3739,7 @@
       <c r="B95" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="C95" s="11" t="s">
+      <c r="C95" s="17" t="s">
         <v>182</v>
       </c>
       <c r="D95" s="8"/>
@@ -3739,10 +3747,10 @@
     </row>
     <row r="96" customHeight="1" spans="1:5">
       <c r="A96" s="6"/>
-      <c r="B96" s="22" t="s">
+      <c r="B96" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="C96" s="11" t="s">
+      <c r="C96" s="17" t="s">
         <v>184</v>
       </c>
       <c r="D96" s="8"/>
@@ -3753,7 +3761,7 @@
       <c r="B97" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="C97" s="11" t="s">
+      <c r="C97" s="17" t="s">
         <v>186</v>
       </c>
       <c r="D97" s="8"/>
@@ -3764,7 +3772,7 @@
       <c r="B98" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="C98" s="11" t="s">
+      <c r="C98" s="17" t="s">
         <v>188</v>
       </c>
       <c r="D98" s="8"/>
@@ -3775,7 +3783,7 @@
       <c r="B99" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="C99" s="15" t="s">
+      <c r="C99" s="16" t="s">
         <v>190</v>
       </c>
       <c r="D99" s="8"/>
@@ -3786,7 +3794,7 @@
       <c r="B100" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="C100" s="15" t="s">
+      <c r="C100" s="16" t="s">
         <v>192</v>
       </c>
       <c r="D100" s="8"/>
@@ -3797,7 +3805,7 @@
       <c r="B101" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="C101" s="15" t="s">
+      <c r="C101" s="16" t="s">
         <v>194</v>
       </c>
       <c r="D101" s="8"/>
@@ -3808,7 +3816,7 @@
       <c r="B102" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="C102" s="15" t="s">
+      <c r="C102" s="16" t="s">
         <v>196</v>
       </c>
       <c r="D102" s="8"/>
@@ -3819,7 +3827,7 @@
       <c r="B103" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="C103" s="15" t="s">
+      <c r="C103" s="16" t="s">
         <v>198</v>
       </c>
       <c r="D103" s="8"/>
@@ -3830,7 +3838,7 @@
       <c r="B104" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="C104" s="15" t="s">
+      <c r="C104" s="16" t="s">
         <v>200</v>
       </c>
       <c r="D104" s="8"/>
@@ -3841,7 +3849,7 @@
       <c r="B105" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="C105" s="15" t="s">
+      <c r="C105" s="16" t="s">
         <v>202</v>
       </c>
       <c r="D105" s="8"/>
@@ -3857,13 +3865,13 @@
       <c r="E106" s="8"/>
     </row>
     <row r="107" customHeight="1" spans="1:5">
-      <c r="A107" s="23" t="s">
+      <c r="A107" s="25" t="s">
         <v>204</v>
       </c>
-      <c r="B107" s="24" t="s">
+      <c r="B107" s="26" t="s">
         <v>205</v>
       </c>
-      <c r="C107" s="20" t="s">
+      <c r="C107" s="22" t="s">
         <v>206</v>
       </c>
       <c r="D107" s="8"/>
@@ -3871,10 +3879,10 @@
     </row>
     <row r="108" customHeight="1" spans="1:5">
       <c r="A108" s="6"/>
-      <c r="B108" s="24" t="s">
+      <c r="B108" s="26" t="s">
         <v>207</v>
       </c>
-      <c r="C108" s="20" t="s">
+      <c r="C108" s="22" t="s">
         <v>208</v>
       </c>
       <c r="D108" s="8"/>
@@ -3882,10 +3890,10 @@
     </row>
     <row r="109" customHeight="1" spans="1:5">
       <c r="A109" s="6"/>
-      <c r="B109" s="24" t="s">
+      <c r="B109" s="26" t="s">
         <v>209</v>
       </c>
-      <c r="C109" s="20" t="s">
+      <c r="C109" s="22" t="s">
         <v>210</v>
       </c>
       <c r="D109" s="8"/>
@@ -3893,23 +3901,23 @@
     </row>
     <row r="110" customHeight="1" spans="1:5">
       <c r="A110" s="6"/>
-      <c r="B110" s="24" t="s">
+      <c r="B110" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="C110" s="20" t="s">
+      <c r="C110" s="22" t="s">
         <v>212</v>
       </c>
       <c r="D110" s="8"/>
       <c r="E110" s="8"/>
     </row>
     <row r="111" customHeight="1" spans="1:5">
-      <c r="A111" s="23" t="s">
+      <c r="A111" s="25" t="s">
         <v>213</v>
       </c>
-      <c r="B111" s="25" t="s">
+      <c r="B111" s="27" t="s">
         <v>214</v>
       </c>
-      <c r="C111" s="20" t="s">
+      <c r="C111" s="22" t="s">
         <v>215</v>
       </c>
       <c r="D111" s="8"/>
@@ -3917,10 +3925,10 @@
     </row>
     <row r="112" customHeight="1" spans="1:5">
       <c r="A112" s="6"/>
-      <c r="B112" s="25" t="s">
+      <c r="B112" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="C112" s="17" t="s">
+      <c r="C112" s="19" t="s">
         <v>217</v>
       </c>
       <c r="D112" s="8"/>
@@ -3928,23 +3936,23 @@
     </row>
     <row r="113" customHeight="1" spans="1:5">
       <c r="A113" s="6"/>
-      <c r="B113" s="25" t="s">
+      <c r="B113" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="C113" s="17" t="s">
+      <c r="C113" s="19" t="s">
         <v>219</v>
       </c>
       <c r="D113" s="8"/>
       <c r="E113" s="8"/>
     </row>
     <row r="114" customHeight="1" spans="1:5">
-      <c r="A114" s="23" t="s">
+      <c r="A114" s="25" t="s">
         <v>220</v>
       </c>
-      <c r="B114" s="26" t="s">
+      <c r="B114" s="28" t="s">
         <v>221</v>
       </c>
-      <c r="C114" s="20" t="s">
+      <c r="C114" s="22" t="s">
         <v>222</v>
       </c>
       <c r="D114" s="8"/>
@@ -3952,34 +3960,34 @@
     </row>
     <row r="115" customHeight="1" spans="1:5">
       <c r="A115" s="6"/>
-      <c r="B115" s="26" t="s">
+      <c r="B115" s="28" t="s">
         <v>223</v>
       </c>
-      <c r="C115" s="17" t="s">
+      <c r="C115" s="19" t="s">
         <v>198</v>
       </c>
       <c r="D115" s="8"/>
       <c r="E115" s="8"/>
     </row>
     <row r="116" customHeight="1" spans="1:5">
-      <c r="A116" s="23" t="s">
+      <c r="A116" s="25" t="s">
         <v>224</v>
       </c>
-      <c r="B116" s="27" t="s">
+      <c r="B116" s="29" t="s">
         <v>225</v>
       </c>
-      <c r="C116" s="17" t="s">
+      <c r="C116" s="19" t="s">
         <v>226</v>
       </c>
       <c r="D116" s="8"/>
       <c r="E116" s="8"/>
     </row>
     <row r="117" customHeight="1" spans="1:5">
-      <c r="A117" s="16"/>
-      <c r="B117" s="27" t="s">
+      <c r="A117" s="18"/>
+      <c r="B117" s="29" t="s">
         <v>227</v>
       </c>
-      <c r="C117" s="20" t="s">
+      <c r="C117" s="22" t="s">
         <v>228</v>
       </c>
       <c r="D117" s="8"/>
@@ -3987,10 +3995,10 @@
     </row>
     <row r="118" customHeight="1" spans="1:5">
       <c r="A118" s="6"/>
-      <c r="B118" s="27" t="s">
+      <c r="B118" s="29" t="s">
         <v>229</v>
       </c>
-      <c r="C118" s="20" t="s">
+      <c r="C118" s="22" t="s">
         <v>230</v>
       </c>
       <c r="D118" s="8"/>
@@ -3998,10 +4006,10 @@
     </row>
     <row r="119" customHeight="1" spans="1:5">
       <c r="A119" s="6"/>
-      <c r="B119" s="27" t="s">
+      <c r="B119" s="29" t="s">
         <v>231</v>
       </c>
-      <c r="C119" s="17" t="s">
+      <c r="C119" s="19" t="s">
         <v>232</v>
       </c>
       <c r="D119" s="8"/>
@@ -4009,10 +4017,10 @@
     </row>
     <row r="120" customHeight="1" spans="1:5">
       <c r="A120" s="6"/>
-      <c r="B120" s="27" t="s">
+      <c r="B120" s="29" t="s">
         <v>233</v>
       </c>
-      <c r="C120" s="20" t="s">
+      <c r="C120" s="22" t="s">
         <v>234</v>
       </c>
       <c r="D120" s="8"/>
@@ -4020,23 +4028,23 @@
     </row>
     <row r="121" customHeight="1" spans="1:5">
       <c r="A121" s="6"/>
-      <c r="B121" s="27" t="s">
+      <c r="B121" s="29" t="s">
         <v>235</v>
       </c>
-      <c r="C121" s="17" t="s">
+      <c r="C121" s="19" t="s">
         <v>236</v>
       </c>
       <c r="D121" s="8"/>
       <c r="E121" s="8"/>
     </row>
     <row r="122" customHeight="1" spans="1:5">
-      <c r="A122" s="23" t="s">
+      <c r="A122" s="25" t="s">
         <v>237</v>
       </c>
-      <c r="B122" s="28" t="s">
+      <c r="B122" s="30" t="s">
         <v>238</v>
       </c>
-      <c r="C122" s="17" t="s">
+      <c r="C122" s="19" t="s">
         <v>239</v>
       </c>
       <c r="D122" s="8"/>
@@ -4044,10 +4052,10 @@
     </row>
     <row r="123" customHeight="1" spans="1:5">
       <c r="A123" s="6"/>
-      <c r="B123" s="28" t="s">
+      <c r="B123" s="30" t="s">
         <v>240</v>
       </c>
-      <c r="C123" s="17" t="s">
+      <c r="C123" s="19" t="s">
         <v>241</v>
       </c>
       <c r="D123" s="8"/>
@@ -4067,10 +4075,10 @@
       <c r="B125" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="C125" s="20" t="s">
+      <c r="C125" s="22" t="s">
         <v>244</v>
       </c>
-      <c r="D125" s="17" t="s">
+      <c r="D125" s="19" t="s">
         <v>245</v>
       </c>
       <c r="E125" s="8"/>
@@ -4080,10 +4088,10 @@
       <c r="B126" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="C126" s="20" t="s">
+      <c r="C126" s="22" t="s">
         <v>247</v>
       </c>
-      <c r="D126" s="17" t="s">
+      <c r="D126" s="19" t="s">
         <v>245</v>
       </c>
       <c r="E126" s="8"/>
@@ -4093,10 +4101,10 @@
       <c r="B127" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="C127" s="20" t="s">
+      <c r="C127" s="22" t="s">
         <v>249</v>
       </c>
-      <c r="D127" s="17" t="s">
+      <c r="D127" s="19" t="s">
         <v>250</v>
       </c>
       <c r="E127" s="8"/>
@@ -4106,10 +4114,10 @@
       <c r="B128" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="C128" s="20" t="s">
+      <c r="C128" s="22" t="s">
         <v>252</v>
       </c>
-      <c r="D128" s="17" t="s">
+      <c r="D128" s="19" t="s">
         <v>250</v>
       </c>
       <c r="E128" s="8"/>
@@ -4119,10 +4127,10 @@
       <c r="B129" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="C129" s="20" t="s">
+      <c r="C129" s="22" t="s">
         <v>254</v>
       </c>
-      <c r="D129" s="17" t="s">
+      <c r="D129" s="19" t="s">
         <v>250</v>
       </c>
       <c r="E129" s="8"/>
@@ -4132,7 +4140,7 @@
       <c r="B130" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="C130" s="20" t="s">
+      <c r="C130" s="22" t="s">
         <v>256</v>
       </c>
       <c r="D130" s="8"/>
@@ -4143,10 +4151,10 @@
       <c r="B131" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="C131" s="20" t="s">
+      <c r="C131" s="22" t="s">
         <v>258</v>
       </c>
-      <c r="D131" s="17" t="s">
+      <c r="D131" s="19" t="s">
         <v>259</v>
       </c>
       <c r="E131" s="8"/>
@@ -4156,7 +4164,7 @@
       <c r="B132" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="C132" s="17" t="s">
+      <c r="C132" s="19" t="s">
         <v>261</v>
       </c>
       <c r="D132" s="8"/>
@@ -4167,7 +4175,7 @@
       <c r="B133" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="C133" s="20" t="s">
+      <c r="C133" s="22" t="s">
         <v>263</v>
       </c>
       <c r="D133" s="8"/>
@@ -4175,10 +4183,10 @@
     </row>
     <row r="134" customHeight="1" spans="1:5">
       <c r="A134" s="6"/>
-      <c r="B134" s="16" t="s">
+      <c r="B134" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="C134" s="17" t="s">
+      <c r="C134" s="19" t="s">
         <v>265</v>
       </c>
       <c r="D134" s="8"/>
@@ -4190,330 +4198,330 @@
       </c>
     </row>
     <row r="136" customHeight="1" spans="1:3">
-      <c r="A136" s="18" t="s">
+      <c r="A136" s="20" t="s">
         <v>267</v>
       </c>
-      <c r="B136" s="19" t="s">
+      <c r="B136" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="C136" s="29" t="s">
+      <c r="C136" s="31" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="137" customHeight="1" spans="2:3">
-      <c r="B137" s="19" t="s">
+      <c r="B137" s="21" t="s">
         <v>270</v>
       </c>
-      <c r="C137" s="29" t="s">
+      <c r="C137" s="31" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="138" customHeight="1" spans="2:4">
-      <c r="B138" s="19" t="s">
+      <c r="B138" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C138" s="29" t="s">
+      <c r="C138" s="31" t="s">
         <v>273</v>
       </c>
-      <c r="D138" s="19" t="s">
+      <c r="D138" s="21" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="139" customHeight="1" spans="2:3">
-      <c r="B139" s="19" t="s">
+      <c r="B139" s="21" t="s">
         <v>275</v>
       </c>
-      <c r="C139" s="29" t="s">
+      <c r="C139" s="31" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="140" customHeight="1" spans="2:3">
-      <c r="B140" s="19" t="s">
+      <c r="B140" s="21" t="s">
         <v>277</v>
       </c>
-      <c r="C140" s="29" t="s">
+      <c r="C140" s="31" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="141" customHeight="1" spans="2:4">
-      <c r="B141" s="19" t="s">
+      <c r="B141" s="21" t="s">
         <v>279</v>
       </c>
-      <c r="C141" s="29" t="s">
+      <c r="C141" s="31" t="s">
         <v>280</v>
       </c>
-      <c r="D141" s="19" t="s">
+      <c r="D141" s="21" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="142" customHeight="1" spans="1:3">
-      <c r="A142" s="30" t="s">
+      <c r="A142" s="32" t="s">
         <v>281</v>
       </c>
-      <c r="B142" s="19" t="s">
+      <c r="B142" s="21" t="s">
         <v>282</v>
       </c>
-      <c r="C142" s="29" t="s">
+      <c r="C142" s="31" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="143" customHeight="1" spans="2:3">
-      <c r="B143" s="19" t="s">
+      <c r="B143" s="21" t="s">
         <v>284</v>
       </c>
-      <c r="C143" s="29" t="s">
+      <c r="C143" s="31" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="144" customHeight="1" spans="2:4">
-      <c r="B144" s="19" t="s">
+      <c r="B144" s="21" t="s">
         <v>286</v>
       </c>
-      <c r="C144" s="29" t="s">
+      <c r="C144" s="31" t="s">
         <v>287</v>
       </c>
-      <c r="D144" s="19" t="s">
+      <c r="D144" s="21" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="145" customHeight="1" spans="2:3">
-      <c r="B145" s="19" t="s">
+      <c r="B145" s="21" t="s">
         <v>288</v>
       </c>
-      <c r="C145" s="31" t="s">
+      <c r="C145" s="33" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="146" customHeight="1" spans="2:3">
-      <c r="B146" s="19" t="s">
+      <c r="B146" s="21" t="s">
         <v>290</v>
       </c>
-      <c r="C146" s="31" t="s">
+      <c r="C146" s="33" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="147" customHeight="1" spans="1:3">
-      <c r="A147" s="30" t="s">
+      <c r="A147" s="32" t="s">
         <v>292</v>
       </c>
-      <c r="B147" s="19" t="s">
+      <c r="B147" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="C147" s="29" t="s">
+      <c r="C147" s="31" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="148" customHeight="1" spans="2:3">
-      <c r="B148" s="19" t="s">
+      <c r="B148" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="C148" s="29" t="s">
+      <c r="C148" s="31" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="149" customHeight="1" spans="2:3">
-      <c r="B149" s="19" t="s">
+      <c r="B149" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="C149" s="29" t="s">
+      <c r="C149" s="31" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="150" customHeight="1" spans="2:3">
-      <c r="B150" s="19" t="s">
+      <c r="B150" s="21" t="s">
         <v>299</v>
       </c>
-      <c r="C150" s="31" t="s">
+      <c r="C150" s="33" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="151" customHeight="1" spans="2:3">
-      <c r="B151" s="19" t="s">
+      <c r="B151" s="21" t="s">
         <v>301</v>
       </c>
-      <c r="C151" s="29" t="s">
+      <c r="C151" s="31" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="152" customHeight="1" spans="2:3">
-      <c r="B152" s="19" t="s">
+      <c r="B152" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="C152" s="31" t="s">
+      <c r="C152" s="33" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="153" customHeight="1" spans="1:3">
-      <c r="A153" s="30" t="s">
+      <c r="A153" s="32" t="s">
         <v>305</v>
       </c>
-      <c r="B153" s="19" t="s">
+      <c r="B153" s="21" t="s">
         <v>306</v>
       </c>
-      <c r="C153" s="29" t="s">
+      <c r="C153" s="31" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="154" customHeight="1" spans="2:3">
-      <c r="B154" s="19" t="s">
+      <c r="B154" s="21" t="s">
         <v>308</v>
       </c>
-      <c r="C154" s="29" t="s">
+      <c r="C154" s="31" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="155" customHeight="1" spans="2:3">
-      <c r="B155" s="19" t="s">
+      <c r="B155" s="21" t="s">
         <v>310</v>
       </c>
-      <c r="C155" s="29" t="s">
+      <c r="C155" s="31" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="156" customHeight="1" spans="2:3">
-      <c r="B156" s="19" t="s">
+      <c r="B156" s="21" t="s">
         <v>312</v>
       </c>
-      <c r="C156" s="29" t="s">
+      <c r="C156" s="31" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="157" customHeight="1" spans="2:3">
-      <c r="B157" s="19" t="s">
+      <c r="B157" s="21" t="s">
         <v>314</v>
       </c>
-      <c r="C157" s="29" t="s">
+      <c r="C157" s="31" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="158" customHeight="1" spans="2:3">
-      <c r="B158" s="19" t="s">
+      <c r="B158" s="21" t="s">
         <v>316</v>
       </c>
-      <c r="C158" s="29" t="s">
+      <c r="C158" s="31" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="159" customHeight="1" spans="2:3">
-      <c r="B159" s="19" t="s">
+      <c r="B159" s="21" t="s">
         <v>318</v>
       </c>
-      <c r="C159" s="29" t="s">
+      <c r="C159" s="31" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="160" customHeight="1" spans="1:3">
-      <c r="A160" s="30" t="s">
+      <c r="A160" s="32" t="s">
         <v>320</v>
       </c>
-      <c r="B160" s="19" t="s">
+      <c r="B160" s="21" t="s">
         <v>321</v>
       </c>
-      <c r="C160" s="29" t="s">
+      <c r="C160" s="31" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="161" customHeight="1" spans="2:3">
-      <c r="B161" s="19" t="s">
+      <c r="B161" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="C161" s="29" t="s">
+      <c r="C161" s="31" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="162" customHeight="1" spans="2:3">
-      <c r="B162" s="19" t="s">
+      <c r="B162" s="21" t="s">
         <v>325</v>
       </c>
-      <c r="C162" s="29" t="s">
+      <c r="C162" s="31" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="163" customHeight="1" spans="2:3">
-      <c r="B163" s="19" t="s">
+      <c r="B163" s="21" t="s">
         <v>327</v>
       </c>
-      <c r="C163" s="31" t="s">
+      <c r="C163" s="33" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="164" customHeight="1" spans="1:3">
-      <c r="A164" s="30" t="s">
+      <c r="A164" s="32" t="s">
         <v>329</v>
       </c>
-      <c r="B164" s="19" t="s">
+      <c r="B164" s="21" t="s">
         <v>330</v>
       </c>
-      <c r="C164" s="29" t="s">
+      <c r="C164" s="31" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="165" customHeight="1" spans="2:3">
-      <c r="B165" s="19" t="s">
+      <c r="B165" s="21" t="s">
         <v>332</v>
       </c>
-      <c r="C165" s="31" t="s">
+      <c r="C165" s="33" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="166" customHeight="1" spans="2:3">
-      <c r="B166" s="19" t="s">
+      <c r="B166" s="21" t="s">
         <v>334</v>
       </c>
-      <c r="C166" s="31" t="s">
+      <c r="C166" s="33" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="167" customHeight="1" spans="2:2">
-      <c r="B167" s="32" t="s">
+      <c r="B167" s="34" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="168" customHeight="1" spans="2:3">
-      <c r="B168" s="18" t="s">
+      <c r="B168" s="20" t="s">
         <v>337</v>
       </c>
-      <c r="C168" s="29" t="s">
+      <c r="C168" s="31" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="169" customHeight="1" spans="2:3">
-      <c r="B169" s="18" t="s">
+      <c r="B169" s="20" t="s">
         <v>339</v>
       </c>
-      <c r="C169" s="29" t="s">
+      <c r="C169" s="31" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="170" customHeight="1" spans="2:3">
-      <c r="B170" s="18" t="s">
+      <c r="B170" s="20" t="s">
         <v>341</v>
       </c>
-      <c r="C170" s="29" t="s">
+      <c r="C170" s="31" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="171" customHeight="1" spans="2:3">
-      <c r="B171" s="18" t="s">
+      <c r="B171" s="20" t="s">
         <v>343</v>
       </c>
-      <c r="C171" s="29" t="s">
+      <c r="C171" s="31" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="172" customHeight="1" spans="2:3">
-      <c r="B172" s="19" t="s">
+      <c r="B172" s="21" t="s">
         <v>345</v>
       </c>
-      <c r="C172" s="31" t="s">
+      <c r="C172" s="33" t="s">
         <v>346</v>
       </c>
     </row>
     <row r="173" customHeight="1" spans="2:3">
-      <c r="B173" s="19" t="s">
+      <c r="B173" s="21" t="s">
         <v>347</v>
       </c>
-      <c r="C173" s="29" t="s">
+      <c r="C173" s="31" t="s">
         <v>348</v>
       </c>
     </row>

</xml_diff>